<commit_message>
paper run 2026-10-29 18:05
</commit_message>
<xml_diff>
--- a/reports/2026-10-29.xlsx
+++ b/reports/2026-10-29.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,49 @@
       </c>
       <c r="K2" t="n">
         <v>3.9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-29T14:56:15.863931+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.00126</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>4.26</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +593,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +603,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -590,7 +633,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.9</v>
+        <v>8.16</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +643,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3.9</v>
+        <v>8.16</v>
       </c>
     </row>
     <row r="8">
@@ -630,7 +673,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4263.149999999999</v>
+        <v>4267.409999999999</v>
       </c>
     </row>
     <row r="12">
@@ -681,16 +724,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>115.52</v>
+        <v>226.67</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="16">
@@ -700,13 +743,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>117.68</v>
+        <v>479.62</v>
       </c>
       <c r="E16" t="n">
         <v>3.9</v>
@@ -722,7 +765,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -732,7 +775,7 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>115.52</v>
+        <v>189.22</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -741,7 +784,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -751,23 +794,35 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>117.68</v>
+        <v>115.52</v>
       </c>
       <c r="E19" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>172.72</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -777,33 +832,33 @@
         <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>233.2</v>
+        <v>228.83</v>
       </c>
       <c r="E21" t="n">
-        <v>3.9</v>
+        <v>8.16</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
+          <t>По цене входа</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>115.52</v>
+        <v>361.94</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -812,71 +867,78 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>117.68</v>
+        <v>344.35</v>
       </c>
       <c r="E24" t="n">
-        <v>3.9</v>
+        <v>8.16</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>477.46</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>228.83</v>
+      </c>
+      <c r="E27" t="n">
+        <v>8.16</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" t="n">
-        <v>3.9</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По окнам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -898,23 +960,23 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>3.9</v>
+        <v>8.16</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -936,7 +998,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -946,120 +1008,206 @@
         <v>1</v>
       </c>
       <c r="D35" t="n">
+        <v>4.26</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
         <v>3.9</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
         <v>3.9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>4.26</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>3.9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>8.16</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="n">
+        <v>8.16</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>4.26</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" t="n">
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
         <v>3.9</v>
       </c>
     </row>

</xml_diff>